<commit_message>
Uittredepunt invoer op scenario-niveau toepassen (#88)
* Start gemaakt

* tussenstand

* Expanding fixed

* Tussenstand

* Start afronden figuur

* Tussenstand

* Finished

* Finished
</commit_message>
<xml_diff>
--- a/geoprob_pipe/cmd_app/parameter_input/parameter_input_template.xlsx
+++ b/geoprob_pipe/cmd_app/parameter_input/parameter_input_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP\git_clones\GeoProb-Pipe\GeoProb-PipeV4\GeoProb-Pipe\geoprob_pipe\cmd_app\parameter_input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7058583F-D206-4937-8667-AE521B8F8933}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{465FE280-A6B2-48B4-B01C-3FE10854F2E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="725" xr2:uid="{4072986C-855A-4E04-BDA4-92C994E74780}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="725" activeTab="2" xr2:uid="{4072986C-855A-4E04-BDA4-92C994E74780}"/>
   </bookViews>
   <sheets>
     <sheet name="Geohydrologisch model" sheetId="1" r:id="rId1"/>
@@ -104,9 +104,6 @@
   </si>
   <si>
     <t xml:space="preserve">De integer referentie naar de scope (bijvoorbeeld vak_id). Bij traject, niks invullen. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alleen invullen bij scope 'vak'. Indien van toepassing op alle scenario's: niks invullen. Anders naam van ondergrondscenario invullen. </t>
   </si>
   <si>
     <t>Het type distributie. Opties zijn 'deterministic', 'log_normal', 'normal', 'cdf_curve' en 'anders'. De laatste geldt enkel voor de buitenwaterstand.</t>
@@ -316,6 +313,9 @@
   </si>
   <si>
     <t xml:space="preserve">Correlatie op trajectniveau. Getal tussen 0 en 1, waarbij 1 volledig gecorreleerd. GeoProb-Pipe hanteert standaard, 0 wanneer je geen correlatie opgeeft. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alleen invullen bij scope 'vak' of 'uittredepunt'. Indien van toepassing op alle scenario's: niks invullen. Anders naam van ondergrondscenario invullen. Wanneer de scope 'uittredepunt' is, geldt gewoon de kans dit gespecificeerd is voor het vak. </t>
   </si>
 </sst>
 </file>
@@ -872,7 +872,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -880,13 +880,13 @@
         <v>12</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -914,10 +914,10 @@
         <v>0</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>13</v>
@@ -951,7 +951,7 @@
         <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>11</v>
@@ -965,7 +965,7 @@
         <v>8</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>9</v>
@@ -979,7 +979,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>4</v>
@@ -16017,36 +16017,36 @@
         <v>15</v>
       </c>
       <c r="E1" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="G1" s="8" t="s">
+      <c r="H1" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="H1" s="8" t="s">
-        <v>31</v>
-      </c>
       <c r="I1" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="126.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B2" s="16" t="s">
         <v>17</v>
@@ -16055,13 +16055,13 @@
         <v>18</v>
       </c>
       <c r="D2" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="E2" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="16" t="s">
-        <v>20</v>
-      </c>
       <c r="F2" s="16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G2" s="16" t="s">
         <v>16</v>
@@ -16070,16 +16070,16 @@
         <v>16</v>
       </c>
       <c r="I2" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J2" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K2" s="16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L2" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M2" s="16"/>
     </row>
@@ -16100,19 +16100,19 @@
         <v>9</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I3" s="9"/>
       <c r="J3" s="9"/>
       <c r="K3" s="9"/>
       <c r="L3" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M3" s="9" t="s">
         <v>9</v>
@@ -16132,31 +16132,31 @@
         <v>3</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F4" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="G4" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="H4" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="I4" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="J4" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="J4" s="10" t="s">
-        <v>66</v>
-      </c>
       <c r="K4" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -16176,18 +16176,18 @@
   <sheetData>
     <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="C1" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="C1" s="21" t="s">
-        <v>58</v>
-      </c>
     </row>
     <row r="2" spans="1:3" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B2" s="22"/>
       <c r="C2" s="22"/>
@@ -16197,18 +16197,18 @@
         <v>9</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="24" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C4" s="24" t="s">
         <v>5</v>
@@ -16231,20 +16231,20 @@
   <sheetData>
     <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="28" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="C1" s="28" t="s">
         <v>83</v>
-      </c>
-      <c r="C1" s="28" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="51" x14ac:dyDescent="0.25">
       <c r="A2" s="29"/>
       <c r="B2" s="29"/>
       <c r="C2" s="29" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -16255,18 +16255,18 @@
         <v>9</v>
       </c>
       <c r="C3" s="30" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="31" t="s">
+        <v>84</v>
+      </c>
+      <c r="B4" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="B4" s="31" t="s">
+      <c r="C4" s="31" t="s">
         <v>86</v>
-      </c>
-      <c r="C4" s="31" t="s">
-        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -16291,63 +16291,63 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="17" t="s">
-        <v>39</v>
+      <c r="C1" s="17" t="s">
+        <v>42</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="D1" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="F1" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="G1" s="17" t="s">
-        <v>44</v>
-      </c>
     </row>
     <row r="2" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
       <c r="E2" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="1:7" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="G2" s="18"/>
-    </row>
-    <row r="3" spans="1:7" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="B3" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="F3" s="18" t="s">
+      <c r="G3" s="18" t="s">
         <v>53</v>
-      </c>
-      <c r="G3" s="18" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -16422,26 +16422,26 @@
   <sheetData>
     <row r="1" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="25" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B1" s="26" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
-        <v>77</v>
+      <c r="B2" s="26" t="s">
+        <v>78</v>
       </c>
-      <c r="B2" s="26" t="s">
+    </row>
+    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="25" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="25" t="s">
-        <v>80</v>
-      </c>
       <c r="B3" s="26" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>